<commit_message>
Macro permite mismo código a Insumo y Papelería
</commit_message>
<xml_diff>
--- a/app/assets/TiposGastos.xlsx
+++ b/app/assets/TiposGastos.xlsx
@@ -1,123 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-27405" yWindow="2115" windowWidth="21600" windowHeight="11775" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Hoja1" state="visible" r:id="rId4"/>
+    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja1'!$A$1:$B$24</definedName>
+  </definedNames>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
-  <si>
-    <t>CODIGO</t>
-  </si>
-  <si>
-    <t>TIPO_GASTO</t>
-  </si>
-  <si>
-    <t>Agua</t>
-  </si>
-  <si>
-    <t>Alimentos</t>
-  </si>
-  <si>
-    <t>Artículos De Limpieza</t>
-  </si>
-  <si>
-    <t>Bolsas</t>
-  </si>
-  <si>
-    <t>Energía Eléctrica</t>
-  </si>
-  <si>
-    <t>Equipo de Cómputo Menor</t>
-  </si>
-  <si>
-    <t>Equipo Menor</t>
-  </si>
-  <si>
-    <t>Extintores y Protección Civil</t>
-  </si>
-  <si>
-    <t>Hospedaje</t>
-  </si>
-  <si>
-    <t>Impuesto Hospedaje</t>
-  </si>
-  <si>
-    <t>Licencias y Permisos</t>
-  </si>
-  <si>
-    <t>Medicamentos</t>
-  </si>
-  <si>
-    <t>No Deducibles</t>
-  </si>
-  <si>
-    <t>Otros</t>
-  </si>
-  <si>
-    <t>Papelería</t>
-  </si>
-  <si>
-    <t>Paquetería y Mensajería</t>
-  </si>
-  <si>
-    <t>Pasajes y Taxis</t>
-  </si>
-  <si>
-    <t>Publicidad</t>
-  </si>
-  <si>
-    <t>Recolección De Basura</t>
-  </si>
-  <si>
-    <t>Servicio de Agua</t>
-  </si>
-  <si>
-    <t>Trámites</t>
-  </si>
-  <si>
-    <t>Trasportación</t>
-  </si>
-  <si>
-    <t>Vigilancia</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="4">
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color theme="1"/>
-      <family val="2"/>
+      <sz val="11"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
       <sz val="11"/>
-      <name val="Aptos Narrow"/>
     </font>
     <font>
+      <name val="Aptos Narrow"/>
       <sz val="11"/>
-      <name val="Aptos Narrow"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <color rgb="FF000000"/>
       <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="5">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -213,51 +139,110 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -582,214 +567,300 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C24"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B27"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="21.285714285714285" customWidth="1"/>
-    <col min="2" max="2" width="23.285714285714285" customWidth="1"/>
-    <col min="3" max="24" width="13.571428571428571" customWidth="1"/>
+    <col width="21.33203125" customWidth="1" min="1" max="1"/>
+    <col width="23.33203125" customWidth="1" min="2" max="2"/>
+    <col width="13.5546875" customWidth="1" min="3" max="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CODIGO</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>TIPO_GASTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>601007</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Insumos</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>601003</v>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Energía Eléctrica</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>601004</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Teléfono</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>601005</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Servicio de Agua</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>601006</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Artículos De Limpieza</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>601007</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Papelería</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>601008</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Equipo Menor</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
         <v>601009</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Agua</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>601010</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Recolección De Basura</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>601011</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Medicamentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>601013</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Bolsas</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>601014</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>601102</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Publicidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n">
+        <v>601123</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Trámites</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n">
+        <v>601124</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Licencias y Permisos</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n">
+        <v>601145</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Extintores y Protección Civil</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="n">
+        <v>601146</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Paquetería y Mensajería</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>601151</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Gasolina</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="n">
+        <v>601153</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Trasportación</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="n">
+        <v>601154</v>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Hospedaje</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
         <v>601157</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
-        <v>601006</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
-        <v>601013</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="5">
-        <v>601003</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Alimentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>601158</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Pasajes y Taxis</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n">
+        <v>601159</v>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Impuesto Hospedaje</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>601173</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Vigilancia</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
         <v>601180</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
-        <v>601008</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
-        <v>601145</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="7">
-        <v>601154</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="7">
-        <v>601159</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="7">
-        <v>601124</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
-        <v>601011</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="7">
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Equipo de Cómputo Menor</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="n">
         <v>601264</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="7">
-        <v>601014</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
-        <v>601007</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="7">
-        <v>601146</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="3">
-        <v>601158</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="3">
-        <v>601102</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="3">
-        <v>601010</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="9">
-        <v>601005</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="7">
-        <v>601123</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="7">
-        <v>601153</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="3">
-        <v>601173</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>24</v>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>No Deducibles</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:B24">
-    <sortState ref="A1:B24">
-      <sortCondition ref="B2:B24"/>
+    <sortState ref="A2:B27">
+      <sortCondition ref="A1:A24"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>